<commit_message>
add new field for comm and fill row
</commit_message>
<xml_diff>
--- a/tests/outputs/errors.xlsx
+++ b/tests/outputs/errors.xlsx
@@ -36,7 +36,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="0078FF66"/>
         <bgColor rgb="0078FF66"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFB979"/>
+        <bgColor rgb="00FFB979"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,9 +115,7 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -197,7 +201,7 @@
   <commentList>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>offer_id</t>
+        <t>Offer</t>
       </text>
     </comment>
     <comment ref="C2" authorId="0" shapeId="0">
@@ -508,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -578,10 +582,58 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>